<commit_message>
Remove Job ID tracker field
</commit_message>
<xml_diff>
--- a/templates/linc_tracker_template.xlsx
+++ b/templates/linc_tracker_template.xlsx
@@ -2,9 +2,9 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Instructions" sheetId="1" r:id="R511c435c7542450c"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Input" sheetId="2" r:id="Rffeb645a9d024a95"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Applications" sheetId="3" r:id="R765e00dc6c8240ea"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Instructions" sheetId="1" r:id="Ra52c4462c59e417d"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Input" sheetId="2" r:id="Re6274d793e9c4b34"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Applications" sheetId="3" r:id="R6e8686af94ef45b2"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -461,8 +461,8 @@
 </file>
 
 <file path=xl/tables/table2.xml><?xml version="1.0" encoding="utf-8"?>
-<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="2" name="ApplicationsTable" displayName="ApplicationsTable" ref="A1:K201" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
-  <x:tableColumns count="11">
+<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="2" name="ApplicationsTable" displayName="ApplicationsTable" ref="A1:J201" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
+  <x:tableColumns count="10">
     <x:tableColumn id="1" name="Date Applied"/>
     <x:tableColumn id="2" name="Company"/>
     <x:tableColumn id="3" name="Job Title"/>
@@ -473,7 +473,6 @@
     <x:tableColumn id="8" name="Salary Range"/>
     <x:tableColumn id="9" name="Follow-up"/>
     <x:tableColumn id="10" name="Found On"/>
-    <x:tableColumn id="11" name="Job ID"/>
   </x:tableColumns>
   <x:tableStyleInfo name="TableStyleMedium3" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </x:table>
@@ -2270,7 +2269,7 @@
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R1c167f0f0d604e7d"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R6668cba9a0ef4b03"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -2341,9 +2340,7 @@
       <x:c r="J1" s="48" t="str">
         <x:v>Found On</x:v>
       </x:c>
-      <x:c r="K1" s="32" t="str">
-        <x:v>Job ID</x:v>
-      </x:c>
+      <x:c r="K1"/>
     </x:row>
     <x:row r="2">
       <x:c r="A2" s="51" t="n"/>
@@ -4789,7 +4786,7 @@
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R7401508ca14743b4"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R8e3eb234fa4a4c88"/>
   </x:tableParts>
 </x:worksheet>
 </file>
</xml_diff>